<commit_message>
Updated the html and did a claude sweep to clean code
</commit_message>
<xml_diff>
--- a/assets/Nav Menu Hierarchy.xlsx
+++ b/assets/Nav Menu Hierarchy.xlsx
@@ -516,9 +516,9 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100DF7F6D8D091AD84397AA73254F26B17C" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f5e30f53b7e8d7360a477d47f8134cdf">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="36f5b453-a8e9-40b9-a45f-257b18f04cb0" xmlns:ns3="4779a3b6-8a29-4c94-9c5d-04d1bd5f6895" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9bd3516cd0b2dc71ea34f05ac331eefe" ns2:_="" ns3:_="">
-    <xsd:import namespace="36f5b453-a8e9-40b9-a45f-257b18f04cb0"/>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C99AD71693B3704D82D2E324E7E5DD96" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ce35fd7b5dca0422a804940b0f421bdf">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="50f0a267-9740-4b53-ae1e-1471dce1ad05" xmlns:ns3="4779a3b6-8a29-4c94-9c5d-04d1bd5f6895" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9f32bb5d09d4fca25ac291f2d897d828" ns2:_="" ns3:_="">
+    <xsd:import namespace="50f0a267-9740-4b53-ae1e-1471dce1ad05"/>
     <xsd:import namespace="4779a3b6-8a29-4c94-9c5d-04d1bd5f6895"/>
     <xsd:element name="properties">
       <xsd:complexType>
@@ -526,16 +526,17 @@
           <xsd:element name="documentManagement">
             <xsd:complexType>
               <xsd:all>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -543,63 +544,68 @@
       </xsd:complexType>
     </xsd:element>
   </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="36f5b453-a8e9-40b9-a45f-257b18f04cb0" elementFormDefault="qualified">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="50f0a267-9740-4b53-ae1e-1471dce1ad05" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="11" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="12" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="13" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="14" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="16" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="35990c56-13cd-4167-abe8-1ed970949a90" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="9" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="35990c56-13cd-4167-abe8-1ed970949a90" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
       <xsd:complexType>
         <xsd:sequence>
           <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
         </xsd:sequence>
       </xsd:complexType>
     </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="18" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+    <xsd:element name="MediaServiceMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="12" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="13" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="17" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note">
           <xsd:maxLength value="255"/>
         </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="18" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="19" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
   </xsd:schema>
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="4779a3b6-8a29-4c94-9c5d-04d1bd5f6895" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="17" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{5c1ddaf0-3448-4125-933d-3af13250601d}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="4779a3b6-8a29-4c94-9c5d-04d1bd5f6895">
+    <xsd:element name="TaxCatchAll" ma:index="10" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{5c1ddaf0-3448-4125-933d-3af13250601d}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="4779a3b6-8a29-4c94-9c5d-04d1bd5f6895">
       <xsd:complexType>
         <xsd:complexContent>
           <xsd:extension base="dms:MultiChoiceLookup">
@@ -719,10 +725,25 @@
 </FormTemplates>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="50f0a267-9740-4b53-ae1e-1471dce1ad05">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="4779a3b6-8a29-4c94-9c5d-04d1bd5f6895" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{50078E8F-E2CE-44AD-BC0A-3F03086EB974}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3ABC18B0-5D82-4DDA-AFB0-14233ED6B6C0}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A49BDE2F-EBC4-436D-9729-D25C30456B48}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{861D1A52-4555-480C-9B7D-6E14DF8EC86E}"/>
 </file>
</xml_diff>